<commit_message>
Add web demo console, data validation and external references, defense scripts
</commit_message>
<xml_diff>
--- a/TEST2.xlsx
+++ b/TEST2.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1950" yWindow="1950" windowWidth="28800" windowHeight="15345" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1 (2)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sheet3" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1 (2)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -682,6 +682,11 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="请选择列表中的数据" error="输入值不在下拉列表中，请重新选择。" type="list" errorStyle="stop">
+      <formula1>"甲,乙"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>